<commit_message>
Criação da ficha Ligma no Obsidian 31-08-2025
</commit_message>
<xml_diff>
--- a/Fichas/Culto de Nidhogg/Ficha Ligma.xlsx
+++ b/Fichas/Culto de Nidhogg/Ficha Ligma.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="12315" activeTab="1"/>
+    <workbookView windowWidth="28800" windowHeight="12315"/>
   </bookViews>
   <sheets>
     <sheet name="Ligma" sheetId="1" r:id="rId1"/>
@@ -1013,7 +1013,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="553" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="187">
   <si>
     <t>Atributos</t>
   </si>
@@ -1382,6 +1382,9 @@
   </si>
   <si>
     <t>+2 Guerra</t>
+  </si>
+  <si>
+    <t>Livros comuns</t>
   </si>
   <si>
     <t>Capacidade</t>
@@ -1579,11 +1582,11 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
     <numFmt numFmtId="176" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="177" formatCode="_-&quot;R$&quot;\ * #,##0_-;\-&quot;R$&quot;\ * #,##0_-;_-&quot;R$&quot;\ * &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="177" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="178" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="179" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="179" formatCode="_-&quot;R$&quot;\ * #,##0_-;\-&quot;R$&quot;\ * #,##0_-;_-&quot;R$&quot;\ * &quot;-&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1622,7 +1625,7 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1633,8 +1636,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF0000FF"/>
       <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1648,24 +1652,24 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
-      <sz val="11"/>
+      <sz val="18"/>
       <color theme="3"/>
       <name val="Aptos Narrow"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
+      <color theme="0"/>
       <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1678,77 +1682,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <i/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Aptos Narrow"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Aptos Narrow"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Aptos Narrow"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color rgb="FF7F7F7F"/>
       <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1764,7 +1700,67 @@
     <font>
       <u/>
       <sz val="11"/>
-      <color rgb="FF0000FF"/>
+      <color rgb="FF800080"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Aptos Narrow"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Aptos Narrow"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1775,17 +1771,17 @@
       <charset val="0"/>
     </font>
     <font>
+      <b/>
+      <sz val="9"/>
+      <name val="Arial"/>
+      <charset val="0"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
       <charset val="0"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="9"/>
-      <name val="Arial"/>
-      <charset val="0"/>
     </font>
     <font>
       <sz val="9"/>
@@ -1826,7 +1822,55 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1838,37 +1882,67 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1886,7 +1960,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1898,37 +1972,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
+        <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1940,67 +1990,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2547,15 +2543,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="thin">
         <color rgb="FF7F7F7F"/>
       </left>
@@ -2571,17 +2558,13 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
       </top>
       <bottom style="double">
-        <color rgb="FF3F3F3F"/>
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -2603,159 +2586,172 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color theme="4"/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
       </top>
       <bottom style="double">
-        <color theme="4"/>
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="40" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="43" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="16" borderId="42" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="44" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="43" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="13" borderId="42" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="44" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="41" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="41" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="40" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="41" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="40" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="38" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="38" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="39" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="39" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="38" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="37" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="179" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -5253,18 +5249,18 @@
       </c>
       <c r="D3" s="27">
         <f ca="1">RANDBETWEEN(1,20)</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E3" s="39">
         <f ca="1">SUM(C3:D3)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G3" s="43" t="s">
         <v>83</v>
       </c>
       <c r="H3" s="44">
         <f ca="1">VLOOKUP(G3,B2:E31,4,FALSE)</f>
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" ht="15.75" spans="2:5">
@@ -5278,11 +5274,11 @@
       </c>
       <c r="D4" s="29">
         <f ca="1" t="shared" ref="D4:D31" si="0">RANDBETWEEN(1,20)</f>
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="E4" s="42">
         <f ca="1" t="shared" ref="E4:E31" si="1">SUM(C4:D4)</f>
-        <v>26</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5" ht="14.25" spans="2:5">
@@ -5296,11 +5292,11 @@
       </c>
       <c r="D5" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="E5" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>24</v>
+        <v>11</v>
       </c>
     </row>
     <row r="6" ht="15" spans="2:5">
@@ -5314,11 +5310,11 @@
       </c>
       <c r="D6" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E6" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="7" ht="14.25" spans="2:5">
@@ -5332,11 +5328,11 @@
       </c>
       <c r="D7" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>18</v>
+        <v>8</v>
       </c>
       <c r="E7" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>26</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" ht="15" spans="2:5">
@@ -5350,11 +5346,11 @@
       </c>
       <c r="D8" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="E8" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>27</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9" ht="14.25" spans="2:5">
@@ -5368,11 +5364,11 @@
       </c>
       <c r="D9" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E9" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" ht="15" spans="2:5">
@@ -5386,11 +5382,11 @@
       </c>
       <c r="D10" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>20</v>
+        <v>4</v>
       </c>
       <c r="E10" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>27</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" ht="14.25" spans="2:5">
@@ -5404,11 +5400,11 @@
       </c>
       <c r="D11" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="E11" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>8</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12" ht="15" spans="2:5">
@@ -5440,11 +5436,11 @@
       </c>
       <c r="D13" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>5</v>
+        <v>18</v>
       </c>
       <c r="E13" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>13</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" ht="15" spans="2:5">
@@ -5458,11 +5454,11 @@
       </c>
       <c r="D14" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E14" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" ht="14.25" spans="2:5">
@@ -5476,11 +5472,11 @@
       </c>
       <c r="D15" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E15" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>27</v>
+        <v>24</v>
       </c>
     </row>
     <row r="16" ht="15" spans="2:5">
@@ -5494,11 +5490,11 @@
       </c>
       <c r="D16" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>17</v>
+        <v>8</v>
       </c>
       <c r="E16" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>24</v>
+        <v>15</v>
       </c>
     </row>
     <row r="17" ht="14.25" spans="2:5">
@@ -5512,11 +5508,11 @@
       </c>
       <c r="D17" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E17" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>21</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18" ht="15" spans="2:5">
@@ -5530,11 +5526,11 @@
       </c>
       <c r="D18" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E18" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="19" ht="14.25" spans="2:5">
@@ -5548,11 +5544,11 @@
       </c>
       <c r="D19" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>1</v>
+        <v>16</v>
       </c>
       <c r="E19" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="20" ht="15" spans="2:5">
@@ -5566,11 +5562,11 @@
       </c>
       <c r="D20" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="E20" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>10</v>
+        <v>25</v>
       </c>
     </row>
     <row r="21" ht="14.25" spans="2:5">
@@ -5584,11 +5580,11 @@
       </c>
       <c r="D21" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E21" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>13</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" ht="15" spans="2:5">
@@ -5602,11 +5598,11 @@
       </c>
       <c r="D22" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E22" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="23" ht="14.25" spans="2:5">
@@ -5620,11 +5616,11 @@
       </c>
       <c r="D23" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E23" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24" ht="30" spans="2:5">
@@ -5638,11 +5634,11 @@
       </c>
       <c r="D24" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E24" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>16</v>
+        <v>21</v>
       </c>
     </row>
     <row r="25" ht="14.25" spans="2:5">
@@ -5656,11 +5652,11 @@
       </c>
       <c r="D25" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="26" ht="30" spans="2:5">
@@ -5674,11 +5670,11 @@
       </c>
       <c r="D26" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>1</v>
+        <v>13</v>
       </c>
       <c r="E26" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>16</v>
+        <v>28</v>
       </c>
     </row>
     <row r="27" ht="14.25" spans="2:5">
@@ -5692,11 +5688,11 @@
       </c>
       <c r="D27" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E27" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="28" ht="15" spans="2:5">
@@ -5710,11 +5706,11 @@
       </c>
       <c r="D28" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>17</v>
+        <v>7</v>
       </c>
       <c r="E28" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>25</v>
+        <v>15</v>
       </c>
     </row>
     <row r="29" ht="14.25" spans="2:5">
@@ -5728,11 +5724,11 @@
       </c>
       <c r="D29" s="27">
         <f ca="1" t="shared" si="0"/>
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="E29" s="39">
         <f ca="1" t="shared" si="1"/>
-        <v>26</v>
+        <v>22</v>
       </c>
     </row>
     <row r="30" ht="15" spans="2:5">
@@ -5746,11 +5742,11 @@
       </c>
       <c r="D30" s="29">
         <f ca="1" t="shared" si="0"/>
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="E30" s="42">
         <f ca="1" t="shared" si="1"/>
-        <v>27</v>
+        <v>21</v>
       </c>
     </row>
     <row r="31" ht="15" spans="2:5">
@@ -5764,11 +5760,11 @@
       </c>
       <c r="D31" s="49">
         <f ca="1" t="shared" si="0"/>
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E31" s="44">
         <f ca="1" t="shared" si="1"/>
-        <v>33</v>
+        <v>18</v>
       </c>
     </row>
     <row r="32" ht="14.25"/>
@@ -5789,7 +5785,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="B1:H35"/>
+  <dimension ref="A1:H35"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="7"/>
   <cols>
     <col min="2" max="2" width="23.2833333333333" customWidth="1"/>
@@ -5817,7 +5813,10 @@
       </c>
       <c r="H2" s="36"/>
     </row>
-    <row r="3" ht="14.25" spans="2:8">
+    <row r="3" ht="14.25" spans="1:8">
+      <c r="A3">
+        <v>1</v>
+      </c>
       <c r="B3" s="68" t="s">
         <v>88</v>
       </c>
@@ -5838,7 +5837,10 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" ht="15" spans="2:8">
+    <row r="4" ht="15" spans="1:8">
+      <c r="A4">
+        <v>1</v>
+      </c>
       <c r="B4" s="30" t="s">
         <v>90</v>
       </c>
@@ -5859,7 +5861,10 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" ht="14.25" spans="2:8">
+    <row r="5" ht="14.25" spans="1:8">
+      <c r="A5">
+        <v>1</v>
+      </c>
       <c r="B5" s="68" t="s">
         <v>91</v>
       </c>
@@ -5880,7 +5885,10 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" ht="15" spans="2:8">
+    <row r="6" ht="15" spans="1:8">
+      <c r="A6">
+        <v>2</v>
+      </c>
       <c r="B6" s="30" t="s">
         <v>93</v>
       </c>
@@ -5901,7 +5909,10 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" ht="15" spans="2:8">
+    <row r="7" ht="15" spans="1:8">
+      <c r="A7">
+        <v>3</v>
+      </c>
       <c r="B7" s="68" t="s">
         <v>94</v>
       </c>
@@ -5922,7 +5933,10 @@
         <v>15</v>
       </c>
     </row>
-    <row r="8" ht="15.75" spans="2:5">
+    <row r="8" ht="15.75" spans="1:5">
+      <c r="A8">
+        <v>4</v>
+      </c>
       <c r="B8" s="30" t="s">
         <v>95</v>
       </c>
@@ -5937,7 +5951,10 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" ht="14.25" spans="2:5">
+    <row r="9" ht="14.25" spans="1:5">
+      <c r="A9">
+        <v>5</v>
+      </c>
       <c r="B9" s="68" t="s">
         <v>96</v>
       </c>
@@ -5952,7 +5969,10 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" ht="15" spans="2:5">
+    <row r="10" ht="15" spans="1:5">
+      <c r="A10">
+        <v>6</v>
+      </c>
       <c r="B10" s="30" t="s">
         <v>97</v>
       </c>
@@ -5967,7 +5987,10 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" ht="14.25" spans="2:5">
+    <row r="11" ht="14.25" spans="1:5">
+      <c r="A11">
+        <v>7</v>
+      </c>
       <c r="B11" s="68" t="s">
         <v>98</v>
       </c>
@@ -5982,7 +6005,10 @@
         <v>90</v>
       </c>
     </row>
-    <row r="12" ht="15" spans="2:5">
+    <row r="12" ht="15" spans="1:5">
+      <c r="A12">
+        <v>8</v>
+      </c>
       <c r="B12" s="30" t="s">
         <v>99</v>
       </c>
@@ -5997,7 +6023,10 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" ht="14.25" spans="2:5">
+    <row r="13" ht="14.25" spans="1:5">
+      <c r="A13">
+        <v>9</v>
+      </c>
       <c r="B13" s="68" t="s">
         <v>100</v>
       </c>
@@ -6012,7 +6041,10 @@
         <v>90</v>
       </c>
     </row>
-    <row r="14" ht="15" spans="2:5">
+    <row r="14" ht="15" spans="1:5">
+      <c r="A14">
+        <v>10</v>
+      </c>
       <c r="B14" s="30" t="s">
         <v>101</v>
       </c>
@@ -6027,7 +6059,10 @@
         <v>90</v>
       </c>
     </row>
-    <row r="15" ht="14.25" spans="2:5">
+    <row r="15" ht="14.25" spans="1:5">
+      <c r="A15">
+        <v>10</v>
+      </c>
       <c r="B15" s="68" t="s">
         <v>102</v>
       </c>
@@ -6464,19 +6499,25 @@
       </c>
     </row>
     <row r="18" ht="14.25" spans="2:9">
-      <c r="B18" s="38"/>
+      <c r="B18" s="38" t="s">
+        <v>123</v>
+      </c>
       <c r="C18" s="55"/>
       <c r="D18" s="55"/>
-      <c r="E18" s="27"/>
-      <c r="F18" s="27"/>
+      <c r="E18" s="27">
+        <v>3</v>
+      </c>
+      <c r="F18" s="27">
+        <v>0.1</v>
+      </c>
       <c r="G18" s="27">
         <f t="shared" ref="G18:G21" si="0">PRODUCT(E18:F18)</f>
-        <v>0</v>
+        <v>0.3</v>
       </c>
       <c r="H18" s="27"/>
       <c r="I18" s="39">
         <f t="shared" ref="I18:I21" si="1">PRODUCT(H18,E18)</f>
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="19" ht="15" spans="2:9">
@@ -6530,11 +6571,11 @@
     <row r="22" ht="15"/>
     <row r="23" ht="15.75" spans="2:4">
       <c r="B23" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="C23" s="57">
         <f>SUM(G17:G21,F9:F13,F4:F5)</f>
-        <v>13.1</v>
+        <v>13.4</v>
       </c>
       <c r="D23" s="2">
         <f>Ligma!C3*3</f>
@@ -6543,7 +6584,7 @@
     </row>
     <row r="24" ht="14.25" spans="2:4">
       <c r="B24" s="58" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C24" s="59">
         <f>Ligma!C3*10</f>
@@ -6553,7 +6594,7 @@
     </row>
     <row r="25" ht="15.75" spans="2:4">
       <c r="B25" s="7" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C25" s="61" t="str">
         <f>IF(C23&gt;D23,"Sobrecarga","Sem Penalidade")</f>
@@ -6606,19 +6647,19 @@
     <row r="1" ht="14.25"/>
     <row r="2" ht="15" customHeight="1" spans="2:16">
       <c r="B2" s="24" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C2" s="25" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D2" s="25" t="s">
         <v>1</v>
       </c>
       <c r="E2" s="25" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F2" s="25" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G2" s="25" t="s">
         <v>41</v>
@@ -6627,31 +6668,31 @@
         <v>24</v>
       </c>
       <c r="I2" s="25" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J2" s="25" t="s">
         <v>82</v>
       </c>
       <c r="K2" s="33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L2" s="33" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="M2" s="34" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="O2" s="35" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="P2" s="36"/>
     </row>
     <row r="3" ht="14.25" spans="2:16">
       <c r="B3" s="26" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D3" s="27">
         <f>VLOOKUP(C3,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -6673,13 +6714,13 @@
         <v>8</v>
       </c>
       <c r="K3" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L3" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M3" s="37" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O3" s="38" t="s">
         <v>34</v>
@@ -6690,10 +6731,10 @@
     </row>
     <row r="4" ht="15" spans="2:16">
       <c r="B4" s="28" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C4" s="29" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D4" s="29">
         <f>VLOOKUP(C4,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -6715,13 +6756,13 @@
         <v>7</v>
       </c>
       <c r="K4" s="29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L4" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="M4" s="40" t="s">
         <v>139</v>
-      </c>
-      <c r="M4" s="40" t="s">
-        <v>138</v>
       </c>
       <c r="O4" s="41" t="s">
         <v>60</v>
@@ -6732,10 +6773,10 @@
     </row>
     <row r="5" ht="15" spans="2:16">
       <c r="B5" s="26" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D5" s="27">
         <f>VLOOKUP(C5,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -6757,13 +6798,13 @@
         <v>8</v>
       </c>
       <c r="K5" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L5" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M5" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="O5" s="43" t="s">
         <v>74</v>
@@ -6774,10 +6815,10 @@
     </row>
     <row r="6" ht="16.5" spans="2:13">
       <c r="B6" s="28" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D6" s="29">
         <f>VLOOKUP(C6,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -6799,21 +6840,21 @@
         <v>7</v>
       </c>
       <c r="K6" s="29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L6" s="29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M6" s="40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1" spans="2:16">
       <c r="B7" s="26" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D7" s="27">
         <f>VLOOKUP(C7,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -6835,25 +6876,25 @@
         <v>8</v>
       </c>
       <c r="K7" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L7" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M7" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="O7" s="35" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="P7" s="36"/>
     </row>
     <row r="8" ht="15" customHeight="1" spans="2:16">
       <c r="B8" s="28" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D8" s="29">
         <f>VLOOKUP(C8,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -6875,13 +6916,13 @@
         <v>15</v>
       </c>
       <c r="K8" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="L8" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="M8" s="40" t="s">
         <v>139</v>
-      </c>
-      <c r="L8" s="29" t="s">
-        <v>139</v>
-      </c>
-      <c r="M8" s="40" t="s">
-        <v>138</v>
       </c>
       <c r="O8" s="38" t="s">
         <v>4</v>
@@ -6893,10 +6934,10 @@
     </row>
     <row r="9" ht="15" spans="2:16">
       <c r="B9" s="26" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D9" s="27">
         <f>VLOOKUP(C9,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -6918,13 +6959,13 @@
         <v>13</v>
       </c>
       <c r="K9" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="L9" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="L9" s="27" t="s">
-        <v>138</v>
-      </c>
       <c r="M9" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="O9" s="41" t="s">
         <v>9</v>
@@ -6936,10 +6977,10 @@
     </row>
     <row r="10" ht="15" spans="2:16">
       <c r="B10" s="28" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D10" s="29">
         <f>VLOOKUP(C10,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -6961,13 +7002,13 @@
         <v>7</v>
       </c>
       <c r="K10" s="29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L10" s="29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M10" s="40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="O10" s="38" t="s">
         <v>10</v>
@@ -6979,10 +7020,10 @@
     </row>
     <row r="11" ht="15" spans="2:16">
       <c r="B11" s="26" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D11" s="27">
         <f>VLOOKUP(C11,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7004,13 +7045,13 @@
         <v>7</v>
       </c>
       <c r="K11" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L11" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M11" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="O11" s="41" t="s">
         <v>12</v>
@@ -7022,10 +7063,10 @@
     </row>
     <row r="12" ht="15" spans="2:16">
       <c r="B12" s="28" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D12" s="29">
         <f>VLOOKUP(C12,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7047,13 +7088,13 @@
         <v>6</v>
       </c>
       <c r="K12" s="29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L12" s="29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M12" s="40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="O12" s="38" t="s">
         <v>14</v>
@@ -7065,10 +7106,10 @@
     </row>
     <row r="13" ht="15.75" spans="2:16">
       <c r="B13" s="26" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D13" s="27">
         <f>VLOOKUP(C13,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7090,13 +7131,13 @@
         <v>8</v>
       </c>
       <c r="K13" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L13" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M13" s="37" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O13" s="45" t="s">
         <v>16</v>
@@ -7108,10 +7149,10 @@
     </row>
     <row r="14" ht="15.75" spans="2:13">
       <c r="B14" s="28" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D14" s="29">
         <f>VLOOKUP(C14,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7135,21 +7176,21 @@
         <v>17</v>
       </c>
       <c r="K14" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="L14" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="M14" s="40" t="s">
         <v>139</v>
-      </c>
-      <c r="L14" s="29" t="s">
-        <v>139</v>
-      </c>
-      <c r="M14" s="40" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="15" ht="14.25" spans="2:13">
       <c r="B15" s="26" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D15" s="27">
         <f>VLOOKUP(C15,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7171,21 +7212,21 @@
         <v>8</v>
       </c>
       <c r="K15" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L15" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M15" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" ht="15" spans="2:13">
       <c r="B16" s="28" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D16" s="29">
         <f>VLOOKUP(C16,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7207,21 +7248,21 @@
         <v>7</v>
       </c>
       <c r="K16" s="29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L16" s="29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M16" s="40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" ht="14.25" spans="2:13">
       <c r="B17" s="26" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D17" s="27">
         <f>VLOOKUP(C17,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7243,21 +7284,21 @@
         <v>9</v>
       </c>
       <c r="K17" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L17" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M17" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" ht="15" spans="2:13">
       <c r="B18" s="28" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D18" s="29">
         <f>VLOOKUP(C18,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7279,21 +7320,21 @@
         <v>15</v>
       </c>
       <c r="K18" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="L18" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="L18" s="29" t="s">
-        <v>138</v>
-      </c>
       <c r="M18" s="40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="19" ht="14.25" spans="2:13">
       <c r="B19" s="26" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D19" s="27">
         <f>VLOOKUP(C19,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7315,21 +7356,21 @@
         <v>7</v>
       </c>
       <c r="K19" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L19" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="M19" s="37" t="s">
         <v>139</v>
-      </c>
-      <c r="M19" s="37" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="20" ht="15" spans="2:13">
       <c r="B20" s="28" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D20" s="29">
         <f>VLOOKUP(C20,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7351,13 +7392,13 @@
         <v>8</v>
       </c>
       <c r="K20" s="29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L20" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="M20" s="40" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" ht="14.25" spans="2:13">
@@ -7365,7 +7406,7 @@
         <v>83</v>
       </c>
       <c r="C21" s="27" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D21" s="27">
         <f>VLOOKUP(C21,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7387,21 +7428,21 @@
         <v>12</v>
       </c>
       <c r="K21" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="L21" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="L21" s="27" t="s">
-        <v>138</v>
-      </c>
       <c r="M21" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="22" ht="15" spans="2:13">
       <c r="B22" s="28" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C22" s="29" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D22" s="29">
         <f>VLOOKUP(C22,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7425,21 +7466,21 @@
         <v>17</v>
       </c>
       <c r="K22" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="L22" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="M22" s="40" t="s">
         <v>139</v>
-      </c>
-      <c r="L22" s="29" t="s">
-        <v>139</v>
-      </c>
-      <c r="M22" s="40" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="23" ht="14.25" spans="2:13">
       <c r="B23" s="26" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C23" s="27" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D23" s="27">
         <f>VLOOKUP(C23,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7461,21 +7502,21 @@
         <v>11</v>
       </c>
       <c r="K23" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L23" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="M23" s="37" t="s">
         <v>139</v>
-      </c>
-      <c r="M23" s="37" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="24" ht="15" spans="2:13">
       <c r="B24" s="28" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C24" s="29" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D24" s="29">
         <f>VLOOKUP(C24,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7497,21 +7538,21 @@
         <v>15</v>
       </c>
       <c r="K24" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="L24" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="M24" s="40" t="s">
         <v>139</v>
-      </c>
-      <c r="L24" s="29" t="s">
-        <v>139</v>
-      </c>
-      <c r="M24" s="40" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="25" ht="14.25" spans="2:13">
       <c r="B25" s="26" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D25" s="27">
         <f>VLOOKUP(C25,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7533,21 +7574,21 @@
         <v>15</v>
       </c>
       <c r="K25" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="L25" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="M25" s="37" t="s">
         <v>139</v>
-      </c>
-      <c r="L25" s="27" t="s">
-        <v>139</v>
-      </c>
-      <c r="M25" s="37" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="26" ht="15" spans="2:13">
       <c r="B26" s="30" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C26" s="29" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D26" s="29">
         <f>VLOOKUP(C26,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7569,21 +7610,21 @@
         <v>15</v>
       </c>
       <c r="K26" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="L26" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="M26" s="40" t="s">
         <v>139</v>
-      </c>
-      <c r="L26" s="29" t="s">
-        <v>139</v>
-      </c>
-      <c r="M26" s="40" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="27" ht="14.25" spans="2:13">
       <c r="B27" s="26" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D27" s="27">
         <f>VLOOKUP(C27,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7607,21 +7648,21 @@
         <v>15</v>
       </c>
       <c r="K27" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="L27" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="L27" s="27" t="s">
-        <v>138</v>
-      </c>
       <c r="M27" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="28" ht="15" spans="2:13">
       <c r="B28" s="28" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C28" s="29" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D28" s="29">
         <f>VLOOKUP(C28,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7643,21 +7684,21 @@
         <v>8</v>
       </c>
       <c r="K28" s="29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L28" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="M28" s="40" t="s">
         <v>139</v>
-      </c>
-      <c r="M28" s="40" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="29" ht="14.25" spans="2:13">
       <c r="B29" s="26" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D29" s="27">
         <f>VLOOKUP(C29,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7679,21 +7720,21 @@
         <v>8</v>
       </c>
       <c r="K29" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L29" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M29" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="30" ht="15" spans="2:13">
       <c r="B30" s="28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C30" s="29" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D30" s="29">
         <f>VLOOKUP(C30,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7715,21 +7756,21 @@
         <v>12</v>
       </c>
       <c r="K30" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="L30" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="L30" s="29" t="s">
-        <v>138</v>
-      </c>
       <c r="M30" s="40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="31" ht="14.25" spans="2:13">
       <c r="B31" s="26" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D31" s="27">
         <f>VLOOKUP(C31,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7751,21 +7792,21 @@
         <v>13</v>
       </c>
       <c r="K31" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="L31" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="M31" s="37" t="s">
         <v>139</v>
-      </c>
-      <c r="L31" s="27" t="s">
-        <v>139</v>
-      </c>
-      <c r="M31" s="37" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="32" ht="15" spans="2:13">
       <c r="B32" s="28" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C32" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D32" s="29">
         <f>VLOOKUP(C32,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7787,21 +7828,21 @@
         <v>9</v>
       </c>
       <c r="K32" s="29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L32" s="29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M32" s="40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="33" ht="14.25" spans="2:13">
       <c r="B33" s="31" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C33" s="32" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D33" s="32">
         <f>VLOOKUP(C33,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7823,13 +7864,13 @@
         <v>13</v>
       </c>
       <c r="K33" s="32" t="s">
+        <v>140</v>
+      </c>
+      <c r="L33" s="32" t="s">
         <v>139</v>
       </c>
-      <c r="L33" s="32" t="s">
-        <v>138</v>
-      </c>
       <c r="M33" s="47" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -7870,19 +7911,19 @@
     <row r="1" ht="14.25"/>
     <row r="2" ht="15" customHeight="1" spans="2:16">
       <c r="B2" s="24" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="C2" s="25" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="D2" s="25" t="s">
         <v>1</v>
       </c>
       <c r="E2" s="25" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="F2" s="25" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G2" s="25" t="s">
         <v>41</v>
@@ -7891,31 +7932,31 @@
         <v>24</v>
       </c>
       <c r="I2" s="25" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J2" s="25" t="s">
         <v>82</v>
       </c>
       <c r="K2" s="33" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L2" s="33" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="M2" s="34" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="O2" s="35" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="P2" s="36"/>
     </row>
     <row r="3" ht="14.25" spans="2:16">
       <c r="B3" s="26" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="C3" s="27" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D3" s="27">
         <f>VLOOKUP(C3,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7937,13 +7978,13 @@
         <v>8</v>
       </c>
       <c r="K3" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L3" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M3" s="37" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O3" s="38" t="s">
         <v>34</v>
@@ -7954,10 +7995,10 @@
     </row>
     <row r="4" ht="15" spans="2:16">
       <c r="B4" s="28" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="C4" s="29" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D4" s="29">
         <f>VLOOKUP(C4,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -7979,13 +8020,13 @@
         <v>7</v>
       </c>
       <c r="K4" s="29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L4" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="M4" s="40" t="s">
         <v>139</v>
-      </c>
-      <c r="M4" s="40" t="s">
-        <v>138</v>
       </c>
       <c r="O4" s="41" t="s">
         <v>60</v>
@@ -7996,10 +8037,10 @@
     </row>
     <row r="5" ht="15" spans="2:16">
       <c r="B5" s="26" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C5" s="27" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D5" s="27">
         <f>VLOOKUP(C5,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8021,13 +8062,13 @@
         <v>8</v>
       </c>
       <c r="K5" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L5" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M5" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="O5" s="43" t="s">
         <v>74</v>
@@ -8038,10 +8079,10 @@
     </row>
     <row r="6" ht="16.5" spans="2:13">
       <c r="B6" s="28" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="C6" s="29" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D6" s="29">
         <f>VLOOKUP(C6,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8063,21 +8104,21 @@
         <v>7</v>
       </c>
       <c r="K6" s="29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L6" s="29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M6" s="40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="7" ht="15.75" customHeight="1" spans="2:16">
       <c r="B7" s="26" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C7" s="27" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D7" s="27">
         <f>VLOOKUP(C7,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8099,25 +8140,25 @@
         <v>8</v>
       </c>
       <c r="K7" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L7" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M7" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="O7" s="35" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="P7" s="36"/>
     </row>
     <row r="8" ht="15" customHeight="1" spans="2:16">
       <c r="B8" s="28" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C8" s="29" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D8" s="29">
         <f>VLOOKUP(C8,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8139,13 +8180,13 @@
         <v>15</v>
       </c>
       <c r="K8" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="L8" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="M8" s="40" t="s">
         <v>139</v>
-      </c>
-      <c r="L8" s="29" t="s">
-        <v>139</v>
-      </c>
-      <c r="M8" s="40" t="s">
-        <v>138</v>
       </c>
       <c r="O8" s="38" t="s">
         <v>4</v>
@@ -8157,10 +8198,10 @@
     </row>
     <row r="9" ht="15" spans="2:16">
       <c r="B9" s="26" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="C9" s="27" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D9" s="27">
         <f>VLOOKUP(C9,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8182,13 +8223,13 @@
         <v>13</v>
       </c>
       <c r="K9" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="L9" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="L9" s="27" t="s">
-        <v>138</v>
-      </c>
       <c r="M9" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="O9" s="41" t="s">
         <v>9</v>
@@ -8200,10 +8241,10 @@
     </row>
     <row r="10" ht="15" spans="2:16">
       <c r="B10" s="28" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C10" s="29" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D10" s="29">
         <f>VLOOKUP(C10,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8225,13 +8266,13 @@
         <v>7</v>
       </c>
       <c r="K10" s="29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L10" s="29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M10" s="40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="O10" s="38" t="s">
         <v>10</v>
@@ -8243,10 +8284,10 @@
     </row>
     <row r="11" ht="15" spans="2:16">
       <c r="B11" s="26" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C11" s="27" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D11" s="27">
         <f>VLOOKUP(C11,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8268,13 +8309,13 @@
         <v>7</v>
       </c>
       <c r="K11" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L11" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M11" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="O11" s="41" t="s">
         <v>12</v>
@@ -8286,10 +8327,10 @@
     </row>
     <row r="12" ht="15" spans="2:16">
       <c r="B12" s="28" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C12" s="29" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="D12" s="29">
         <f>VLOOKUP(C12,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8311,13 +8352,13 @@
         <v>6</v>
       </c>
       <c r="K12" s="29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L12" s="29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M12" s="40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="O12" s="38" t="s">
         <v>14</v>
@@ -8329,10 +8370,10 @@
     </row>
     <row r="13" ht="15.75" spans="2:16">
       <c r="B13" s="26" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="C13" s="27" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D13" s="27">
         <f>VLOOKUP(C13,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8354,13 +8395,13 @@
         <v>8</v>
       </c>
       <c r="K13" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L13" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M13" s="37" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="O13" s="45" t="s">
         <v>16</v>
@@ -8372,10 +8413,10 @@
     </row>
     <row r="14" ht="15.75" spans="2:13">
       <c r="B14" s="28" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C14" s="29" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D14" s="29">
         <f>VLOOKUP(C14,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8399,21 +8440,21 @@
         <v>16</v>
       </c>
       <c r="K14" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="L14" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="M14" s="40" t="s">
         <v>139</v>
-      </c>
-      <c r="L14" s="29" t="s">
-        <v>139</v>
-      </c>
-      <c r="M14" s="40" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="15" ht="14.25" spans="2:13">
       <c r="B15" s="26" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C15" s="27" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D15" s="27">
         <f>VLOOKUP(C15,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8435,21 +8476,21 @@
         <v>8</v>
       </c>
       <c r="K15" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L15" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M15" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="16" ht="15" spans="2:13">
       <c r="B16" s="28" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C16" s="29" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D16" s="29">
         <f>VLOOKUP(C16,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8471,21 +8512,21 @@
         <v>7</v>
       </c>
       <c r="K16" s="29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L16" s="29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M16" s="40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="17" ht="14.25" spans="2:13">
       <c r="B17" s="26" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C17" s="27" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D17" s="27">
         <f>VLOOKUP(C17,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8507,21 +8548,21 @@
         <v>9</v>
       </c>
       <c r="K17" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L17" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M17" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="18" ht="15" spans="2:13">
       <c r="B18" s="28" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C18" s="29" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D18" s="29">
         <f>VLOOKUP(C18,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8543,21 +8584,21 @@
         <v>15</v>
       </c>
       <c r="K18" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="L18" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="L18" s="29" t="s">
-        <v>138</v>
-      </c>
       <c r="M18" s="40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="19" ht="14.25" spans="2:13">
       <c r="B19" s="26" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C19" s="27" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="D19" s="27">
         <f>VLOOKUP(C19,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8579,21 +8620,21 @@
         <v>7</v>
       </c>
       <c r="K19" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L19" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="M19" s="37" t="s">
         <v>139</v>
-      </c>
-      <c r="M19" s="37" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="20" ht="15" spans="2:13">
       <c r="B20" s="28" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C20" s="29" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D20" s="29">
         <f>VLOOKUP(C20,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8615,13 +8656,13 @@
         <v>8</v>
       </c>
       <c r="K20" s="29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L20" s="29" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="M20" s="40" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="21" ht="14.25" spans="2:13">
@@ -8629,7 +8670,7 @@
         <v>83</v>
       </c>
       <c r="C21" s="27" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D21" s="27">
         <f>VLOOKUP(C21,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8651,21 +8692,21 @@
         <v>12</v>
       </c>
       <c r="K21" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="L21" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="L21" s="27" t="s">
-        <v>138</v>
-      </c>
       <c r="M21" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="22" ht="15" spans="2:13">
       <c r="B22" s="28" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C22" s="29" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D22" s="29">
         <f>VLOOKUP(C22,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8689,21 +8730,21 @@
         <v>17</v>
       </c>
       <c r="K22" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="L22" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="M22" s="40" t="s">
         <v>139</v>
-      </c>
-      <c r="L22" s="29" t="s">
-        <v>139</v>
-      </c>
-      <c r="M22" s="40" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="23" ht="14.25" spans="2:13">
       <c r="B23" s="26" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C23" s="27" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D23" s="27">
         <f>VLOOKUP(C23,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8725,21 +8766,21 @@
         <v>11</v>
       </c>
       <c r="K23" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L23" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="M23" s="37" t="s">
         <v>139</v>
-      </c>
-      <c r="M23" s="37" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="24" ht="15" spans="2:13">
       <c r="B24" s="28" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C24" s="29" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D24" s="29">
         <f>VLOOKUP(C24,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8761,21 +8802,21 @@
         <v>15</v>
       </c>
       <c r="K24" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="L24" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="M24" s="40" t="s">
         <v>139</v>
-      </c>
-      <c r="L24" s="29" t="s">
-        <v>139</v>
-      </c>
-      <c r="M24" s="40" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="25" ht="14.25" spans="2:13">
       <c r="B25" s="26" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C25" s="27" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D25" s="27">
         <f>VLOOKUP(C25,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8797,21 +8838,21 @@
         <v>15</v>
       </c>
       <c r="K25" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="L25" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="M25" s="37" t="s">
         <v>139</v>
-      </c>
-      <c r="L25" s="27" t="s">
-        <v>139</v>
-      </c>
-      <c r="M25" s="37" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="26" ht="15" spans="2:13">
       <c r="B26" s="30" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C26" s="29" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="D26" s="29">
         <f>VLOOKUP(C26,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8833,21 +8874,21 @@
         <v>15</v>
       </c>
       <c r="K26" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="L26" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="M26" s="40" t="s">
         <v>139</v>
-      </c>
-      <c r="L26" s="29" t="s">
-        <v>139</v>
-      </c>
-      <c r="M26" s="40" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="27" ht="14.25" spans="2:13">
       <c r="B27" s="26" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C27" s="27" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D27" s="27">
         <f>VLOOKUP(C27,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8871,21 +8912,21 @@
         <v>15</v>
       </c>
       <c r="K27" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="L27" s="27" t="s">
         <v>139</v>
       </c>
-      <c r="L27" s="27" t="s">
-        <v>138</v>
-      </c>
       <c r="M27" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="28" ht="15" spans="2:13">
       <c r="B28" s="28" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C28" s="29" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D28" s="29">
         <f>VLOOKUP(C28,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8907,21 +8948,21 @@
         <v>8</v>
       </c>
       <c r="K28" s="29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L28" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="M28" s="40" t="s">
         <v>139</v>
-      </c>
-      <c r="M28" s="40" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="29" ht="14.25" spans="2:13">
       <c r="B29" s="26" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C29" s="27" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D29" s="27">
         <f>VLOOKUP(C29,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8943,21 +8984,21 @@
         <v>8</v>
       </c>
       <c r="K29" s="27" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L29" s="27" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M29" s="37" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="30" ht="15" spans="2:13">
       <c r="B30" s="28" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C30" s="29" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="D30" s="29">
         <f>VLOOKUP(C30,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -8979,21 +9020,21 @@
         <v>12</v>
       </c>
       <c r="K30" s="29" t="s">
+        <v>140</v>
+      </c>
+      <c r="L30" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="L30" s="29" t="s">
-        <v>138</v>
-      </c>
       <c r="M30" s="40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="31" ht="14.25" spans="2:13">
       <c r="B31" s="26" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C31" s="27" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D31" s="27">
         <f>VLOOKUP(C31,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -9015,21 +9056,21 @@
         <v>13</v>
       </c>
       <c r="K31" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="L31" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="M31" s="37" t="s">
         <v>139</v>
-      </c>
-      <c r="L31" s="27" t="s">
-        <v>139</v>
-      </c>
-      <c r="M31" s="37" t="s">
-        <v>138</v>
       </c>
     </row>
     <row r="32" ht="15" spans="2:13">
       <c r="B32" s="28" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C32" s="29" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D32" s="29">
         <f>VLOOKUP(C32,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -9051,21 +9092,21 @@
         <v>9</v>
       </c>
       <c r="K32" s="29" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L32" s="29" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="M32" s="40" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="33" ht="14.25" spans="2:13">
       <c r="B33" s="31" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="C33" s="32" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="D33" s="32">
         <f>VLOOKUP(C33,Ligma!$B$3:$D$8,3,FALSE)</f>
@@ -9087,13 +9128,13 @@
         <v>13</v>
       </c>
       <c r="K33" s="32" t="s">
+        <v>140</v>
+      </c>
+      <c r="L33" s="32" t="s">
         <v>139</v>
       </c>
-      <c r="L33" s="32" t="s">
-        <v>138</v>
-      </c>
       <c r="M33" s="47" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -9126,7 +9167,7 @@
     <row r="1" ht="14.25"/>
     <row r="2" ht="15.75" spans="2:13">
       <c r="B2" s="1" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C2" s="2"/>
       <c r="E2" s="1">
@@ -9136,16 +9177,16 @@
         <v>2</v>
       </c>
       <c r="H2" s="15" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="I2" s="21" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="M2" s="2">
         <f>12+Ligma!D5</f>
@@ -9176,7 +9217,7 @@
         <v>0</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="M3" s="4">
         <v>4</v>
@@ -9206,7 +9247,7 @@
         <v>1</v>
       </c>
       <c r="L4" s="7" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="M4" s="8">
         <v>1</v>
@@ -9322,7 +9363,7 @@
     </row>
     <row r="12" ht="15.75" spans="2:10">
       <c r="B12" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C12" s="2">
         <f>3+Ligma!D5</f>
@@ -9341,7 +9382,7 @@
     </row>
     <row r="13" ht="14.25" spans="2:10">
       <c r="B13" s="3" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C13" s="4">
         <f>SUM(M3:M4)</f>
@@ -9386,13 +9427,13 @@
     </row>
     <row r="16" ht="15.75" spans="2:10">
       <c r="B16" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E16" s="18" t="s">
         <v>82</v>

</xml_diff>